<commit_message>
#3 Transmitter BOM added
</commit_message>
<xml_diff>
--- a/TYPE-C_4K_RECEIVER/Design-Files/BOM/Client-BOM-TYPEC_4KRECEIVER-v1.0.xlsx
+++ b/TYPE-C_4K_RECEIVER/Design-Files/BOM/Client-BOM-TYPEC_4KRECEIVER-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="662">
   <si>
     <t>Component list</t>
   </si>
@@ -1470,9 +1470,6 @@
     <t>C106235</t>
   </si>
   <si>
-    <t>C100044</t>
-  </si>
-  <si>
     <t>C105578</t>
   </si>
   <si>
@@ -1770,9 +1767,6 @@
     <t>40</t>
   </si>
   <si>
-    <t>5000</t>
-  </si>
-  <si>
     <t>0.0011</t>
   </si>
   <si>
@@ -2008,6 +2002,9 @@
   </si>
   <si>
     <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>C95177</t>
   </si>
 </sst>
 </file>
@@ -2406,7 +2403,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2560,6 +2557,9 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="40" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="E3" s="27"/>
       <c r="F3" s="41" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G3" s="29"/>
       <c r="H3" s="30"/>
@@ -3023,34 +3023,34 @@
         <v>376</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>410</v>
       </c>
       <c r="K7" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>561</v>
+      </c>
+      <c r="M7" s="12" t="s">
+        <v>568</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="O7" s="12" t="s">
         <v>566</v>
       </c>
-      <c r="L7" s="12" t="s">
-        <v>562</v>
-      </c>
-      <c r="M7" s="12" t="s">
-        <v>569</v>
-      </c>
-      <c r="N7" s="12" t="s">
+      <c r="P7" s="43" t="s">
         <v>570</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="Q7" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="R7" s="12" t="s">
         <v>567</v>
-      </c>
-      <c r="P7" s="43" t="s">
-        <v>571</v>
-      </c>
-      <c r="Q7" s="12" t="s">
-        <v>572</v>
-      </c>
-      <c r="R7" s="12" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -3078,13 +3078,13 @@
         <v>377</v>
       </c>
       <c r="I8" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L8" s="14">
         <v>2</v>
@@ -3097,7 +3097,7 @@
         <v>11</v>
       </c>
       <c r="O8" s="45" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="P8" s="44">
         <v>2.1</v>
@@ -3133,13 +3133,13 @@
         <v>378</v>
       </c>
       <c r="I9" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J9" s="20" t="s">
         <v>411</v>
       </c>
       <c r="K9" s="20" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L9" s="20">
         <v>2</v>
@@ -3149,10 +3149,10 @@
         <v>10</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O9" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P9" s="44">
         <v>4.0000000000000001E-3</v>
@@ -3188,13 +3188,13 @@
         <v>378</v>
       </c>
       <c r="I10" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J10" s="14" t="s">
         <v>412</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="L10" s="14">
         <v>14</v>
@@ -3204,10 +3204,10 @@
         <v>70</v>
       </c>
       <c r="N10" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O10" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P10" s="44">
         <v>1.1000000000000001E-3</v>
@@ -3243,13 +3243,13 @@
         <v>378</v>
       </c>
       <c r="I11" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J11" s="20" t="s">
         <v>413</v>
       </c>
       <c r="K11" s="20" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L11" s="20">
         <v>1</v>
@@ -3259,13 +3259,13 @@
         <v>5</v>
       </c>
       <c r="N11" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O11" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P11" s="44" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="Q11" s="21">
         <f t="shared" ref="Q11" si="4">P11*N11</f>
@@ -3298,13 +3298,13 @@
         <v>378</v>
       </c>
       <c r="I12" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J12" s="14" t="s">
         <v>414</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="L12" s="14">
         <v>53</v>
@@ -3314,13 +3314,13 @@
         <v>265</v>
       </c>
       <c r="N12" s="14" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="O12" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P12" s="44" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="Q12" s="15">
         <f>P12*N12</f>
@@ -3353,13 +3353,13 @@
         <v>378</v>
       </c>
       <c r="I13" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J13" s="20" t="s">
         <v>415</v>
       </c>
       <c r="K13" s="20" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L13" s="20">
         <v>14</v>
@@ -3369,13 +3369,13 @@
         <v>70</v>
       </c>
       <c r="N13" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O13" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P13" s="44" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="Q13" s="21">
         <f t="shared" ref="Q13" si="6">P13*N13</f>
@@ -3408,13 +3408,13 @@
         <v>379</v>
       </c>
       <c r="I14" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J14" s="14" t="s">
         <v>416</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="L14" s="14">
         <v>2</v>
@@ -3424,13 +3424,13 @@
         <v>10</v>
       </c>
       <c r="N14" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O14" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P14" s="44" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="Q14" s="15">
         <f>P14*N14</f>
@@ -3463,13 +3463,13 @@
         <v>379</v>
       </c>
       <c r="I15" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J15" s="20" t="s">
         <v>417</v>
       </c>
       <c r="K15" s="20" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L15" s="20">
         <v>23</v>
@@ -3482,10 +3482,10 @@
         <v>120</v>
       </c>
       <c r="O15" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P15" s="44" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="Q15" s="21">
         <f t="shared" ref="Q15" si="8">P15*N15</f>
@@ -3518,13 +3518,13 @@
         <v>380</v>
       </c>
       <c r="I16" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J16" s="14" t="s">
         <v>418</v>
       </c>
       <c r="K16" s="14" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L16" s="14">
         <v>3</v>
@@ -3534,13 +3534,13 @@
         <v>15</v>
       </c>
       <c r="N16" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O16" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P16" s="44" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="Q16" s="15">
         <f>P16*N16</f>
@@ -3573,11 +3573,11 @@
         <v>378</v>
       </c>
       <c r="I17" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J17" s="20"/>
       <c r="K17" s="20" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="L17" s="20">
         <v>1</v>
@@ -3587,13 +3587,13 @@
         <v>5</v>
       </c>
       <c r="N17" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O17" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P17" s="44" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="Q17" s="21">
         <f t="shared" ref="Q17" si="10">P17*N17</f>
@@ -3626,13 +3626,13 @@
         <v>378</v>
       </c>
       <c r="I18" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J18" s="14" t="s">
         <v>419</v>
       </c>
       <c r="K18" s="14" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L18" s="14">
         <v>29</v>
@@ -3642,13 +3642,13 @@
         <v>145</v>
       </c>
       <c r="N18" s="14" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="O18" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P18" s="44" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="Q18" s="15">
         <f>P18*N18</f>
@@ -3681,13 +3681,13 @@
         <v>378</v>
       </c>
       <c r="I19" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J19" s="20" t="s">
         <v>420</v>
       </c>
       <c r="K19" s="20" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L19" s="20">
         <v>9</v>
@@ -3697,13 +3697,13 @@
         <v>45</v>
       </c>
       <c r="N19" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O19" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P19" s="44" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="Q19" s="21">
         <f t="shared" ref="Q19" si="12">P19*N19</f>
@@ -3736,13 +3736,13 @@
         <v>380</v>
       </c>
       <c r="I20" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J20" s="14" t="s">
         <v>421</v>
       </c>
       <c r="K20" s="14" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L20" s="14">
         <v>15</v>
@@ -3752,13 +3752,13 @@
         <v>75</v>
       </c>
       <c r="N20" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O20" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P20" s="44" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="Q20" s="15">
         <f>P20*N20</f>
@@ -3791,13 +3791,13 @@
         <v>378</v>
       </c>
       <c r="I21" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J21" s="20" t="s">
         <v>422</v>
       </c>
       <c r="K21" s="20" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="L21" s="20">
         <v>68</v>
@@ -3807,13 +3807,13 @@
         <v>340</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="O21" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P21" s="44" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="Q21" s="21">
         <f t="shared" ref="Q21" si="14">P21*N21</f>
@@ -3846,13 +3846,13 @@
         <v>378</v>
       </c>
       <c r="I22" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J22" s="14" t="s">
         <v>423</v>
       </c>
       <c r="K22" s="14" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="L22" s="14">
         <v>2</v>
@@ -3862,13 +3862,13 @@
         <v>10</v>
       </c>
       <c r="N22" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O22" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P22" s="44" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="Q22" s="15">
         <f>P22*N22</f>
@@ -3901,13 +3901,13 @@
         <v>378</v>
       </c>
       <c r="I23" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J23" s="20" t="s">
         <v>424</v>
       </c>
       <c r="K23" s="20" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L23" s="20">
         <v>3</v>
@@ -3917,13 +3917,13 @@
         <v>15</v>
       </c>
       <c r="N23" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O23" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P23" s="44" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="Q23" s="21">
         <f t="shared" ref="Q23" si="16">P23*N23</f>
@@ -3956,13 +3956,13 @@
         <v>381</v>
       </c>
       <c r="I24" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J24" s="14" t="s">
         <v>425</v>
       </c>
       <c r="K24" s="14" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="L24" s="14">
         <v>3</v>
@@ -3972,13 +3972,13 @@
         <v>15</v>
       </c>
       <c r="N24" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O24" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P24" s="44" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="Q24" s="15">
         <f>P24*N24</f>
@@ -4011,13 +4011,13 @@
         <v>378</v>
       </c>
       <c r="I25" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J25" s="20" t="s">
         <v>414</v>
       </c>
       <c r="K25" s="20" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="L25" s="20">
         <v>4</v>
@@ -4027,13 +4027,13 @@
         <v>20</v>
       </c>
       <c r="N25" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O25" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P25" s="44" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="Q25" s="21">
         <f t="shared" ref="Q25" si="18">P25*N25</f>
@@ -4066,13 +4066,13 @@
         <v>379</v>
       </c>
       <c r="I26" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J26" s="14" t="s">
         <v>426</v>
       </c>
       <c r="K26" s="14" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="L26" s="14">
         <v>1</v>
@@ -4085,10 +4085,10 @@
         <v>10</v>
       </c>
       <c r="O26" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P26" s="44" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="Q26" s="15">
         <f>P26*N26</f>
@@ -4121,13 +4121,13 @@
         <v>379</v>
       </c>
       <c r="I27" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J27" s="20" t="s">
         <v>427</v>
       </c>
       <c r="K27" s="20" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="L27" s="20">
         <v>2</v>
@@ -4140,10 +4140,10 @@
         <v>15</v>
       </c>
       <c r="O27" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P27" s="44" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="Q27" s="21">
         <f t="shared" ref="Q27" si="20">P27*N27</f>
@@ -4176,13 +4176,13 @@
         <v>380</v>
       </c>
       <c r="I28" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="K28" s="14" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="L28" s="14">
         <v>2</v>
@@ -4192,13 +4192,13 @@
         <v>10</v>
       </c>
       <c r="N28" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O28" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P28" s="44" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="Q28" s="15">
         <f>P28*N28</f>
@@ -4231,13 +4231,13 @@
         <v>378</v>
       </c>
       <c r="I29" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J29" s="20" t="s">
         <v>428</v>
       </c>
       <c r="K29" s="20" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L29" s="20">
         <v>4</v>
@@ -4247,13 +4247,13 @@
         <v>20</v>
       </c>
       <c r="N29" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O29" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P29" s="44" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="Q29" s="21">
         <f t="shared" ref="Q29" si="22">P29*N29</f>
@@ -4286,13 +4286,13 @@
         <v>382</v>
       </c>
       <c r="I30" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J30" s="14" t="s">
         <v>429</v>
       </c>
       <c r="K30" s="14" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L30" s="14">
         <v>4</v>
@@ -4302,13 +4302,13 @@
         <v>20</v>
       </c>
       <c r="N30" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O30" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P30" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q30" s="15">
         <f>P30*N30</f>
@@ -4341,13 +4341,13 @@
         <v>379</v>
       </c>
       <c r="I31" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J31" s="20" t="s">
         <v>430</v>
       </c>
       <c r="K31" s="20" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="L31" s="20">
         <v>2</v>
@@ -4357,13 +4357,13 @@
         <v>10</v>
       </c>
       <c r="N31" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O31" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P31" s="44" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="Q31" s="21">
         <f t="shared" ref="Q31" si="24">P31*N31</f>
@@ -4396,13 +4396,13 @@
         <v>378</v>
       </c>
       <c r="I32" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J32" s="14" t="s">
         <v>431</v>
       </c>
       <c r="K32" s="14" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="L32" s="14">
         <v>1</v>
@@ -4412,13 +4412,13 @@
         <v>5</v>
       </c>
       <c r="N32" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O32" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P32" s="44" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="Q32" s="15">
         <f>P32*N32</f>
@@ -4451,13 +4451,13 @@
         <v>378</v>
       </c>
       <c r="I33" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J33" s="46" t="s">
         <v>432</v>
       </c>
       <c r="K33" s="46" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="L33" s="46">
         <v>4</v>
@@ -4470,16 +4470,16 @@
         <v>40</v>
       </c>
       <c r="O33" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P33" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q33" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R33" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -4507,13 +4507,13 @@
         <v>379</v>
       </c>
       <c r="I34" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J34" s="14" t="s">
         <v>433</v>
       </c>
       <c r="K34" s="14" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L34" s="14">
         <v>6</v>
@@ -4523,13 +4523,13 @@
         <v>30</v>
       </c>
       <c r="N34" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O34" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P34" s="44" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="Q34" s="15">
         <f>P34*N34</f>
@@ -4562,13 +4562,13 @@
         <v>379</v>
       </c>
       <c r="I35" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J35" s="46" t="s">
         <v>434</v>
       </c>
       <c r="K35" s="46" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="L35" s="46">
         <v>1</v>
@@ -4578,19 +4578,19 @@
         <v>5</v>
       </c>
       <c r="N35" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O35" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P35" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q35" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R35" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -4618,13 +4618,13 @@
         <v>379</v>
       </c>
       <c r="I36" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J36" s="14" t="s">
         <v>435</v>
       </c>
       <c r="K36" s="14" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="L36" s="14">
         <v>1</v>
@@ -4634,13 +4634,13 @@
         <v>5</v>
       </c>
       <c r="N36" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O36" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P36" s="44" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="Q36" s="15">
         <f>P36*N36</f>
@@ -4673,13 +4673,13 @@
         <v>379</v>
       </c>
       <c r="I37" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J37" s="20" t="s">
         <v>436</v>
       </c>
       <c r="K37" s="20" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="L37" s="20">
         <v>2</v>
@@ -4689,13 +4689,13 @@
         <v>10</v>
       </c>
       <c r="N37" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O37" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P37" s="44" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="Q37" s="21">
         <f t="shared" ref="Q37" si="28">P37*N37</f>
@@ -4728,13 +4728,13 @@
         <v>378</v>
       </c>
       <c r="I38" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J38" s="47" t="s">
         <v>437</v>
       </c>
       <c r="K38" s="47" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L38" s="47">
         <v>1</v>
@@ -4744,19 +4744,19 @@
         <v>5</v>
       </c>
       <c r="N38" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O38" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P38" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q38" s="51" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R38" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -4784,13 +4784,13 @@
         <v>378</v>
       </c>
       <c r="I39" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J39" s="20" t="s">
         <v>438</v>
       </c>
       <c r="K39" s="20" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="L39" s="20">
         <v>2</v>
@@ -4800,13 +4800,13 @@
         <v>10</v>
       </c>
       <c r="N39" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O39" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P39" s="44" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="Q39" s="21">
         <f t="shared" ref="Q39" si="30">P39*N39</f>
@@ -4839,13 +4839,13 @@
         <v>383</v>
       </c>
       <c r="I40" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J40" s="14" t="s">
         <v>439</v>
       </c>
       <c r="K40" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L40" s="14">
         <v>7</v>
@@ -4855,13 +4855,13 @@
         <v>35</v>
       </c>
       <c r="N40" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O40" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P40" s="44" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="Q40" s="15">
         <f>P40*N40</f>
@@ -4894,13 +4894,13 @@
         <v>383</v>
       </c>
       <c r="I41" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J41" s="20" t="s">
         <v>440</v>
       </c>
       <c r="K41" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L41" s="20">
         <v>2</v>
@@ -4910,13 +4910,13 @@
         <v>10</v>
       </c>
       <c r="N41" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O41" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P41" s="44" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="Q41" s="21">
         <f t="shared" ref="Q41" si="32">P41*N41</f>
@@ -4949,13 +4949,13 @@
         <v>384</v>
       </c>
       <c r="I42" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J42" s="14" t="s">
         <v>441</v>
       </c>
       <c r="K42" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L42" s="14">
         <v>2</v>
@@ -4968,10 +4968,10 @@
         <v>20</v>
       </c>
       <c r="O42" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P42" s="44" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="Q42" s="15">
         <f>P42*N42</f>
@@ -5004,13 +5004,13 @@
         <v>384</v>
       </c>
       <c r="I43" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J43" s="20" t="s">
         <v>442</v>
       </c>
       <c r="K43" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L43" s="20">
         <v>2</v>
@@ -5020,13 +5020,13 @@
         <v>10</v>
       </c>
       <c r="N43" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O43" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P43" s="44" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="Q43" s="21">
         <f t="shared" ref="Q43" si="34">P43*N43</f>
@@ -5041,7 +5041,7 @@
         <v>37</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D44" s="14" t="s">
         <v>63</v>
@@ -5059,13 +5059,13 @@
         <v>385</v>
       </c>
       <c r="I44" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J44" s="14" t="s">
         <v>443</v>
       </c>
       <c r="K44" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L44" s="14">
         <v>1</v>
@@ -5075,13 +5075,13 @@
         <v>5</v>
       </c>
       <c r="N44" s="14" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="O44" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P44" s="44" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="Q44" s="15">
         <f>P44*N44</f>
@@ -5114,13 +5114,13 @@
         <v>379</v>
       </c>
       <c r="I45" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J45" s="20" t="s">
         <v>444</v>
       </c>
       <c r="K45" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L45" s="20">
         <v>5</v>
@@ -5130,13 +5130,13 @@
         <v>25</v>
       </c>
       <c r="N45" s="14" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="O45" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P45" s="44" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="Q45" s="21">
         <f t="shared" ref="Q45" si="36">P45*N45</f>
@@ -5169,13 +5169,13 @@
         <v>386</v>
       </c>
       <c r="I46" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J46" s="14" t="s">
         <v>445</v>
       </c>
       <c r="K46" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L46" s="14">
         <v>1</v>
@@ -5185,13 +5185,13 @@
         <v>5</v>
       </c>
       <c r="N46" s="14" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="O46" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P46" s="44" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="Q46" s="15">
         <f>P46*N46</f>
@@ -5215,7 +5215,7 @@
         <v>177</v>
       </c>
       <c r="F47" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G47" s="20" t="s">
         <v>318</v>
@@ -5224,13 +5224,13 @@
         <v>387</v>
       </c>
       <c r="I47" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J47" s="20" t="s">
         <v>446</v>
       </c>
       <c r="K47" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L47" s="20">
         <v>1</v>
@@ -5243,10 +5243,10 @@
         <v>10</v>
       </c>
       <c r="O47" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P47" s="44" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="Q47" s="21">
         <f t="shared" ref="Q47" si="38">P47*N47</f>
@@ -5270,7 +5270,7 @@
         <v>178</v>
       </c>
       <c r="F48" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G48" s="42" t="s">
         <v>255</v>
@@ -5279,13 +5279,13 @@
         <v>388</v>
       </c>
       <c r="I48" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J48" s="14" t="s">
         <v>447</v>
       </c>
       <c r="K48" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L48" s="14">
         <v>1</v>
@@ -5298,10 +5298,10 @@
         <v>6</v>
       </c>
       <c r="O48" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P48" s="44" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="Q48" s="15">
         <f>P48*N48</f>
@@ -5325,7 +5325,7 @@
         <v>179</v>
       </c>
       <c r="F49" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G49" s="20" t="s">
         <v>256</v>
@@ -5334,13 +5334,13 @@
         <v>389</v>
       </c>
       <c r="I49" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J49" s="20" t="s">
         <v>448</v>
       </c>
       <c r="K49" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L49" s="20">
         <v>1</v>
@@ -5350,13 +5350,13 @@
         <v>5</v>
       </c>
       <c r="N49" s="14" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="O49" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P49" s="44" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="Q49" s="21">
         <f t="shared" ref="Q49" si="40">P49*N49</f>
@@ -5380,7 +5380,7 @@
         <v>180</v>
       </c>
       <c r="F50" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G50" s="14" t="s">
         <v>257</v>
@@ -5389,13 +5389,13 @@
         <v>390</v>
       </c>
       <c r="I50" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J50" s="14" t="s">
         <v>449</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="L50" s="14">
         <v>2</v>
@@ -5408,10 +5408,10 @@
         <v>20</v>
       </c>
       <c r="O50" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P50" s="44" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="Q50" s="15">
         <f>P50*N50</f>
@@ -5435,7 +5435,7 @@
         <v>181</v>
       </c>
       <c r="F51" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G51" s="20" t="s">
         <v>319</v>
@@ -5444,13 +5444,13 @@
         <v>390</v>
       </c>
       <c r="I51" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J51" s="20" t="s">
         <v>450</v>
       </c>
       <c r="K51" s="20" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="L51" s="20">
         <v>1</v>
@@ -5460,13 +5460,13 @@
         <v>5</v>
       </c>
       <c r="N51" s="14" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="O51" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P51" s="44" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="Q51" s="21">
         <f t="shared" ref="Q51" si="42">P51*N51</f>
@@ -5490,7 +5490,7 @@
         <v>182</v>
       </c>
       <c r="F52" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G52" s="14" t="s">
         <v>258</v>
@@ -5499,13 +5499,13 @@
         <v>391</v>
       </c>
       <c r="I52" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J52" s="14" t="s">
         <v>451</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="L52" s="14">
         <v>5</v>
@@ -5518,10 +5518,10 @@
         <v>30</v>
       </c>
       <c r="O52" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P52" s="44" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="Q52" s="15">
         <f>P52*N52</f>
@@ -5545,7 +5545,7 @@
         <v>183</v>
       </c>
       <c r="F53" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G53" s="20" t="s">
         <v>320</v>
@@ -5554,13 +5554,13 @@
         <v>390</v>
       </c>
       <c r="I53" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J53" s="20" t="s">
         <v>452</v>
       </c>
       <c r="K53" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L53" s="20">
         <v>2</v>
@@ -5570,13 +5570,13 @@
         <v>10</v>
       </c>
       <c r="N53" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O53" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P53" s="44" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="Q53" s="21">
         <f t="shared" ref="Q53" si="44">P53*N53</f>
@@ -5600,7 +5600,7 @@
         <v>184</v>
       </c>
       <c r="F54" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G54" s="14" t="s">
         <v>321</v>
@@ -5609,13 +5609,13 @@
         <v>390</v>
       </c>
       <c r="I54" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J54" s="14" t="s">
         <v>453</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="L54" s="14">
         <v>1</v>
@@ -5628,10 +5628,10 @@
         <v>10</v>
       </c>
       <c r="O54" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P54" s="44" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="Q54" s="15">
         <f>P54*N54</f>
@@ -5655,7 +5655,7 @@
         <v>185</v>
       </c>
       <c r="F55" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G55" s="20" t="s">
         <v>322</v>
@@ -5664,13 +5664,13 @@
         <v>391</v>
       </c>
       <c r="I55" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J55" s="20" t="s">
         <v>454</v>
       </c>
       <c r="K55" s="20" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="L55" s="20">
         <v>1</v>
@@ -5683,10 +5683,10 @@
         <v>10</v>
       </c>
       <c r="O55" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P55" s="44" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="Q55" s="21">
         <f t="shared" ref="Q55" si="46">P55*N55</f>
@@ -5710,7 +5710,7 @@
         <v>186</v>
       </c>
       <c r="F56" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G56" s="14" t="s">
         <v>259</v>
@@ -5719,13 +5719,13 @@
         <v>392</v>
       </c>
       <c r="I56" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J56" s="14" t="s">
         <v>455</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="L56" s="14">
         <v>1</v>
@@ -5738,10 +5738,10 @@
         <v>10</v>
       </c>
       <c r="O56" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P56" s="44" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="Q56" s="15">
         <f>P56*N56</f>
@@ -5765,7 +5765,7 @@
         <v>187</v>
       </c>
       <c r="F57" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G57" s="20" t="s">
         <v>260</v>
@@ -5774,13 +5774,13 @@
         <v>393</v>
       </c>
       <c r="I57" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J57" s="20" t="s">
         <v>456</v>
       </c>
       <c r="K57" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L57" s="20">
         <v>1</v>
@@ -5790,13 +5790,13 @@
         <v>5</v>
       </c>
       <c r="N57" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O57" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P57" s="44" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="Q57" s="21">
         <f t="shared" ref="Q57" si="48">P57*N57</f>
@@ -5829,13 +5829,13 @@
         <v>394</v>
       </c>
       <c r="I58" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J58" s="14" t="s">
         <v>457</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L58" s="14">
         <v>2</v>
@@ -5845,13 +5845,13 @@
         <v>10</v>
       </c>
       <c r="N58" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O58" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P58" s="44" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="Q58" s="15">
         <f>P58*N58</f>
@@ -5884,13 +5884,13 @@
         <v>378</v>
       </c>
       <c r="I59" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J59" s="20" t="s">
         <v>458</v>
       </c>
       <c r="K59" s="20" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L59" s="20">
         <v>19</v>
@@ -5900,13 +5900,13 @@
         <v>95</v>
       </c>
       <c r="N59" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O59" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P59" s="44" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="Q59" s="21">
         <f t="shared" ref="Q59" si="50">P59*N59</f>
@@ -5939,13 +5939,13 @@
         <v>378</v>
       </c>
       <c r="I60" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J60" s="14" t="s">
         <v>459</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="L60" s="14">
         <v>11</v>
@@ -5955,13 +5955,13 @@
         <v>55</v>
       </c>
       <c r="N60" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O60" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P60" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q60" s="15">
         <f>P60*N60</f>
@@ -5994,13 +5994,13 @@
         <v>378</v>
       </c>
       <c r="I61" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J61" s="20" t="s">
         <v>460</v>
       </c>
       <c r="K61" s="20" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="L61" s="20">
         <v>20</v>
@@ -6010,13 +6010,13 @@
         <v>100</v>
       </c>
       <c r="N61" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O61" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P61" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q61" s="21">
         <f t="shared" ref="Q61" si="52">P61*N61</f>
@@ -6049,13 +6049,13 @@
         <v>378</v>
       </c>
       <c r="I62" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J62" s="14" t="s">
         <v>461</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="L62" s="14">
         <v>4</v>
@@ -6065,13 +6065,13 @@
         <v>20</v>
       </c>
       <c r="N62" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O62" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P62" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q62" s="15">
         <f>P62*N62</f>
@@ -6104,13 +6104,13 @@
         <v>378</v>
       </c>
       <c r="I63" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J63" s="20" t="s">
         <v>462</v>
       </c>
       <c r="K63" s="20" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L63" s="20">
         <v>6</v>
@@ -6120,13 +6120,13 @@
         <v>30</v>
       </c>
       <c r="N63" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O63" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P63" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q63" s="21">
         <f t="shared" ref="Q63" si="54">P63*N63</f>
@@ -6159,13 +6159,13 @@
         <v>378</v>
       </c>
       <c r="I64" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J64" s="14" t="s">
         <v>463</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L64" s="14">
         <v>2</v>
@@ -6175,13 +6175,13 @@
         <v>10</v>
       </c>
       <c r="N64" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O64" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P64" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q64" s="15">
         <f>P64*N64</f>
@@ -6214,13 +6214,13 @@
         <v>395</v>
       </c>
       <c r="I65" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J65" s="20" t="s">
         <v>464</v>
       </c>
       <c r="K65" s="20" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="L65" s="20">
         <v>1</v>
@@ -6230,13 +6230,13 @@
         <v>5</v>
       </c>
       <c r="N65" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O65" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P65" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q65" s="21">
         <f t="shared" ref="Q65" si="56">P65*N65</f>
@@ -6269,13 +6269,13 @@
         <v>378</v>
       </c>
       <c r="I66" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J66" s="14" t="s">
         <v>465</v>
       </c>
       <c r="K66" s="14" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L66" s="14">
         <v>1</v>
@@ -6285,13 +6285,13 @@
         <v>5</v>
       </c>
       <c r="N66" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O66" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P66" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q66" s="15">
         <f>P66*N66</f>
@@ -6324,13 +6324,13 @@
         <v>378</v>
       </c>
       <c r="I67" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J67" s="20" t="s">
         <v>466</v>
       </c>
       <c r="K67" s="20" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="L67" s="20">
         <v>1</v>
@@ -6340,13 +6340,13 @@
         <v>5</v>
       </c>
       <c r="N67" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O67" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P67" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q67" s="21">
         <f t="shared" ref="Q67" si="58">P67*N67</f>
@@ -6379,13 +6379,13 @@
         <v>378</v>
       </c>
       <c r="I68" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J68" s="14" t="s">
         <v>467</v>
       </c>
       <c r="K68" s="14" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="L68" s="14">
         <v>10</v>
@@ -6395,13 +6395,13 @@
         <v>50</v>
       </c>
       <c r="N68" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O68" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P68" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q68" s="15">
         <f>P68*N68</f>
@@ -6434,13 +6434,13 @@
         <v>378</v>
       </c>
       <c r="I69" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J69" s="20" t="s">
         <v>468</v>
       </c>
       <c r="K69" s="20" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="L69" s="20">
         <v>1</v>
@@ -6450,13 +6450,13 @@
         <v>5</v>
       </c>
       <c r="N69" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O69" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P69" s="44" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="Q69" s="21">
         <f t="shared" ref="Q69" si="60">P69*N69</f>
@@ -6489,13 +6489,13 @@
         <v>378</v>
       </c>
       <c r="I70" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J70" s="14" t="s">
         <v>469</v>
       </c>
       <c r="K70" s="14" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="L70" s="14">
         <v>1</v>
@@ -6505,13 +6505,13 @@
         <v>5</v>
       </c>
       <c r="N70" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O70" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P70" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q70" s="15">
         <f>P70*N70</f>
@@ -6544,13 +6544,13 @@
         <v>378</v>
       </c>
       <c r="I71" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J71" s="20" t="s">
         <v>470</v>
       </c>
       <c r="K71" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="L71" s="20">
         <v>1</v>
@@ -6560,13 +6560,13 @@
         <v>5</v>
       </c>
       <c r="N71" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O71" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P71" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q71" s="21">
         <f t="shared" ref="Q71" si="62">P71*N71</f>
@@ -6599,13 +6599,13 @@
         <v>378</v>
       </c>
       <c r="I72" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J72" s="14" t="s">
         <v>471</v>
       </c>
       <c r="K72" s="14" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="L72" s="14">
         <v>1</v>
@@ -6615,13 +6615,13 @@
         <v>5</v>
       </c>
       <c r="N72" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O72" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P72" s="44" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="Q72" s="15">
         <f>P72*N72</f>
@@ -6654,13 +6654,13 @@
         <v>378</v>
       </c>
       <c r="I73" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J73" s="20" t="s">
         <v>472</v>
       </c>
       <c r="K73" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="L73" s="20">
         <v>1</v>
@@ -6670,13 +6670,13 @@
         <v>5</v>
       </c>
       <c r="N73" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O73" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P73" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q73" s="21">
         <f t="shared" ref="Q73" si="64">P73*N73</f>
@@ -6709,13 +6709,13 @@
         <v>378</v>
       </c>
       <c r="I74" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J74" s="47" t="s">
         <v>460</v>
       </c>
       <c r="K74" s="47" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L74" s="47">
         <v>13</v>
@@ -6725,19 +6725,19 @@
         <v>65</v>
       </c>
       <c r="N74" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O74" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P74" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q74" s="51" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R74" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="75" spans="1:18">
@@ -6765,13 +6765,13 @@
         <v>378</v>
       </c>
       <c r="I75" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J75" s="20" t="s">
         <v>473</v>
       </c>
       <c r="K75" s="20" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="L75" s="20">
         <v>1</v>
@@ -6781,13 +6781,13 @@
         <v>5</v>
       </c>
       <c r="N75" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O75" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P75" s="44" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="Q75" s="21">
         <f t="shared" ref="Q75" si="66">P75*N75</f>
@@ -6820,13 +6820,13 @@
         <v>378</v>
       </c>
       <c r="I76" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J76" s="14" t="s">
         <v>474</v>
       </c>
       <c r="K76" s="14" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L76" s="14">
         <v>1</v>
@@ -6836,13 +6836,13 @@
         <v>5</v>
       </c>
       <c r="N76" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O76" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P76" s="44" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="Q76" s="15">
         <f>P76*N76</f>
@@ -6875,13 +6875,13 @@
         <v>378</v>
       </c>
       <c r="I77" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J77" s="20" t="s">
         <v>475</v>
       </c>
       <c r="K77" s="20" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="L77" s="20">
         <v>1</v>
@@ -6891,13 +6891,13 @@
         <v>5</v>
       </c>
       <c r="N77" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O77" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P77" s="44" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="Q77" s="21">
         <f t="shared" ref="Q77" si="68">P77*N77</f>
@@ -6930,13 +6930,13 @@
         <v>378</v>
       </c>
       <c r="I78" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J78" s="14" t="s">
         <v>476</v>
       </c>
       <c r="K78" s="14" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="L78" s="14">
         <v>2</v>
@@ -6946,13 +6946,13 @@
         <v>10</v>
       </c>
       <c r="N78" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O78" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P78" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q78" s="15">
         <f>P78*N78</f>
@@ -6985,13 +6985,13 @@
         <v>378</v>
       </c>
       <c r="I79" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J79" s="47" t="s">
         <v>458</v>
       </c>
       <c r="K79" s="47" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="L79" s="47">
         <v>1</v>
@@ -7001,19 +7001,19 @@
         <v>5</v>
       </c>
       <c r="N79" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O79" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P79" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q79" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R79" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="80" spans="1:18">
@@ -7041,13 +7041,13 @@
         <v>378</v>
       </c>
       <c r="I80" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J80" s="14" t="s">
         <v>477</v>
       </c>
       <c r="K80" s="14" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L80" s="14">
         <v>5</v>
@@ -7057,13 +7057,13 @@
         <v>25</v>
       </c>
       <c r="N80" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O80" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P80" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q80" s="15">
         <f>P80*N80</f>
@@ -7096,13 +7096,13 @@
         <v>378</v>
       </c>
       <c r="I81" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J81" s="20" t="s">
         <v>478</v>
       </c>
       <c r="K81" s="20" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="L81" s="20">
         <v>8</v>
@@ -7112,13 +7112,13 @@
         <v>40</v>
       </c>
       <c r="N81" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O81" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P81" s="44" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="Q81" s="21">
         <f t="shared" ref="Q81" si="71">P81*N81</f>
@@ -7151,13 +7151,13 @@
         <v>378</v>
       </c>
       <c r="I82" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J82" s="14" t="s">
         <v>479</v>
       </c>
       <c r="K82" s="14" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L82" s="14">
         <v>4</v>
@@ -7167,13 +7167,13 @@
         <v>20</v>
       </c>
       <c r="N82" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O82" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P82" s="44" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="Q82" s="15">
         <f>P82*N82</f>
@@ -7206,13 +7206,13 @@
         <v>378</v>
       </c>
       <c r="I83" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J83" s="20" t="s">
         <v>480</v>
       </c>
       <c r="K83" s="20" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="L83" s="20">
         <v>1</v>
@@ -7222,13 +7222,13 @@
         <v>5</v>
       </c>
       <c r="N83" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O83" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P83" s="44" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="Q83" s="21">
         <f t="shared" ref="Q83" si="73">P83*N83</f>
@@ -7261,13 +7261,13 @@
         <v>378</v>
       </c>
       <c r="I84" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J84" s="47" t="s">
         <v>481</v>
       </c>
       <c r="K84" s="47" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="L84" s="47">
         <v>4</v>
@@ -7277,19 +7277,19 @@
         <v>20</v>
       </c>
       <c r="N84" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O84" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P84" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q84" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R84" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="85" spans="1:18">
@@ -7317,13 +7317,13 @@
         <v>378</v>
       </c>
       <c r="I85" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J85" s="20" t="s">
         <v>481</v>
       </c>
       <c r="K85" s="20" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L85" s="20">
         <v>2</v>
@@ -7333,13 +7333,13 @@
         <v>10</v>
       </c>
       <c r="N85" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O85" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P85" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q85" s="21">
         <f t="shared" ref="Q85" si="75">P85*N85</f>
@@ -7372,13 +7372,13 @@
         <v>378</v>
       </c>
       <c r="I86" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J86" s="47" t="s">
         <v>482</v>
       </c>
       <c r="K86" s="47" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="L86" s="47">
         <v>2</v>
@@ -7388,19 +7388,19 @@
         <v>10</v>
       </c>
       <c r="N86" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O86" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P86" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q86" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R86" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="87" spans="1:18">
@@ -7428,13 +7428,13 @@
         <v>378</v>
       </c>
       <c r="I87" s="53" t="s">
+        <v>659</v>
+      </c>
+      <c r="J87" s="20" t="s">
         <v>661</v>
       </c>
-      <c r="J87" s="20" t="s">
-        <v>483</v>
-      </c>
       <c r="K87" s="20" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="L87" s="20">
         <v>1</v>
@@ -7443,16 +7443,18 @@
         <f t="shared" ref="M87" si="76">L87*5</f>
         <v>5</v>
       </c>
-      <c r="N87" s="14" t="s">
-        <v>583</v>
-      </c>
-      <c r="O87" s="45"/>
+      <c r="N87" s="14">
+        <v>100</v>
+      </c>
+      <c r="O87" s="58" t="s">
+        <v>654</v>
+      </c>
       <c r="P87" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q87" s="21">
         <f t="shared" ref="Q87" si="77">P87*N87</f>
-        <v>2.9999999999999996</v>
+        <v>0.06</v>
       </c>
       <c r="R87" s="20"/>
     </row>
@@ -7481,13 +7483,13 @@
         <v>378</v>
       </c>
       <c r="I88" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J88" s="47" t="s">
         <v>460</v>
       </c>
       <c r="K88" s="47" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="L88" s="47">
         <v>14</v>
@@ -7497,19 +7499,19 @@
         <v>70</v>
       </c>
       <c r="N88" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O88" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P88" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q88" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R88" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="89" spans="1:18">
@@ -7537,13 +7539,13 @@
         <v>378</v>
       </c>
       <c r="I89" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J89" s="20" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="K89" s="20" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="L89" s="20">
         <v>1</v>
@@ -7553,13 +7555,13 @@
         <v>5</v>
       </c>
       <c r="N89" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O89" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P89" s="44" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="Q89" s="21">
         <f t="shared" ref="Q89" si="79">P89*N89</f>
@@ -7592,13 +7594,13 @@
         <v>378</v>
       </c>
       <c r="I90" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J90" s="14" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="K90" s="14" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="L90" s="14">
         <v>1</v>
@@ -7608,13 +7610,13 @@
         <v>5</v>
       </c>
       <c r="N90" s="14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="O90" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P90" s="44" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="Q90" s="15">
         <f>P90*N90</f>
@@ -7647,13 +7649,13 @@
         <v>378</v>
       </c>
       <c r="I91" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J91" s="20" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="K91" s="20" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L91" s="20">
         <v>1</v>
@@ -7663,13 +7665,13 @@
         <v>5</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O91" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P91" s="44" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="Q91" s="21">
         <f t="shared" ref="Q91" si="81">P91*N91</f>
@@ -7702,11 +7704,11 @@
         <v>378</v>
       </c>
       <c r="I92" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J92" s="14"/>
       <c r="K92" s="14" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="L92" s="14">
         <v>2</v>
@@ -7716,13 +7718,13 @@
         <v>10</v>
       </c>
       <c r="N92" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O92" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P92" s="44" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="Q92" s="15">
         <f>P92*N92</f>
@@ -7755,13 +7757,13 @@
         <v>378</v>
       </c>
       <c r="I93" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J93" s="47" t="s">
         <v>458</v>
       </c>
       <c r="K93" s="47" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L93" s="47">
         <v>2</v>
@@ -7771,19 +7773,19 @@
         <v>10</v>
       </c>
       <c r="N93" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O93" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P93" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q93" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R93" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="94" spans="1:18">
@@ -7811,13 +7813,13 @@
         <v>378</v>
       </c>
       <c r="I94" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J94" s="14" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="L94" s="14">
         <v>2</v>
@@ -7827,13 +7829,13 @@
         <v>10</v>
       </c>
       <c r="N94" s="14" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="O94" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P94" s="44" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="Q94" s="15">
         <f>P94*N94</f>
@@ -7866,13 +7868,13 @@
         <v>378</v>
       </c>
       <c r="I95" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J95" s="47" t="s">
         <v>458</v>
       </c>
       <c r="K95" s="47" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="L95" s="47">
         <v>2</v>
@@ -7882,19 +7884,19 @@
         <v>10</v>
       </c>
       <c r="N95" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O95" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P95" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q95" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R95" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="96" spans="1:18">
@@ -7922,13 +7924,13 @@
         <v>378</v>
       </c>
       <c r="I96" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J96" s="14" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K96" s="14" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="L96" s="14">
         <v>1</v>
@@ -7938,13 +7940,13 @@
         <v>5</v>
       </c>
       <c r="N96" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O96" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P96" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q96" s="15">
         <f>P96*N96</f>
@@ -7977,11 +7979,11 @@
         <v>378</v>
       </c>
       <c r="I97" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J97" s="20"/>
       <c r="K97" s="20" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="L97" s="20">
         <v>5</v>
@@ -7991,13 +7993,13 @@
         <v>25</v>
       </c>
       <c r="N97" s="14" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O97" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P97" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="Q97" s="21">
         <f t="shared" ref="Q97" si="85">P97*N97</f>
@@ -8030,13 +8032,13 @@
         <v>378</v>
       </c>
       <c r="I98" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J98" s="47" t="s">
         <v>482</v>
       </c>
       <c r="K98" s="47" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L98" s="47">
         <v>1</v>
@@ -8046,19 +8048,19 @@
         <v>5</v>
       </c>
       <c r="N98" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O98" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P98" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q98" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R98" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="99" spans="1:18">
@@ -8086,13 +8088,13 @@
         <v>378</v>
       </c>
       <c r="I99" s="54" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J99" s="46" t="s">
         <v>462</v>
       </c>
       <c r="K99" s="46" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L99" s="46">
         <v>1</v>
@@ -8102,19 +8104,19 @@
         <v>5</v>
       </c>
       <c r="N99" s="47" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="O99" s="48" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P99" s="49" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Q99" s="50" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R99" s="52" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="100" spans="1:18">
@@ -8133,7 +8135,7 @@
         <v>222</v>
       </c>
       <c r="F100" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G100" s="14" t="s">
         <v>265</v>
@@ -8142,13 +8144,13 @@
         <v>396</v>
       </c>
       <c r="I100" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J100" s="14" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="K100" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L100" s="14">
         <v>3</v>
@@ -8161,10 +8163,10 @@
         <v>20</v>
       </c>
       <c r="O100" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P100" s="44" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="Q100" s="15">
         <f>P100*N100</f>
@@ -8197,13 +8199,13 @@
         <v>397</v>
       </c>
       <c r="I101" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J101" s="20" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="K101" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L101" s="20">
         <v>1</v>
@@ -8216,10 +8218,10 @@
         <v>6</v>
       </c>
       <c r="O101" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P101" s="44" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="Q101" s="21">
         <f t="shared" ref="Q101" si="88">P101*N101</f>
@@ -8252,11 +8254,11 @@
         <v>398</v>
       </c>
       <c r="I102" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J102" s="14"/>
       <c r="K102" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L102" s="14">
         <v>1</v>
@@ -8269,10 +8271,10 @@
         <v>6</v>
       </c>
       <c r="O102" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P102" s="44" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="Q102" s="15">
         <f>P102*N102</f>
@@ -8305,13 +8307,13 @@
         <v>380</v>
       </c>
       <c r="I103" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J103" s="20" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="K103" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L103" s="20">
         <v>1</v>
@@ -8324,10 +8326,10 @@
         <v>6</v>
       </c>
       <c r="O103" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P103" s="44" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="Q103" s="21">
         <f t="shared" ref="Q103" si="90">P103*N103</f>
@@ -8360,13 +8362,13 @@
         <v>399</v>
       </c>
       <c r="I104" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J104" s="14" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="K104" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L104" s="14">
         <v>2</v>
@@ -8379,10 +8381,10 @@
         <v>15</v>
       </c>
       <c r="O104" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P104" s="44" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="Q104" s="15">
         <f>P104*N104</f>
@@ -8415,13 +8417,13 @@
         <v>399</v>
       </c>
       <c r="I105" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J105" s="20" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="K105" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L105" s="20">
         <v>1</v>
@@ -8434,10 +8436,10 @@
         <v>6</v>
       </c>
       <c r="O105" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P105" s="44" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="Q105" s="21">
         <f t="shared" ref="Q105" si="92">P105*N105</f>
@@ -8470,13 +8472,13 @@
         <v>400</v>
       </c>
       <c r="I106" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J106" s="14" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="K106" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L106" s="14">
         <v>1</v>
@@ -8489,10 +8491,10 @@
         <v>6</v>
       </c>
       <c r="O106" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P106" s="44" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="Q106" s="15">
         <f>P106*N106</f>
@@ -8525,13 +8527,13 @@
         <v>397</v>
       </c>
       <c r="I107" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J107" s="20" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="K107" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L107" s="20">
         <v>1</v>
@@ -8544,10 +8546,10 @@
         <v>6</v>
       </c>
       <c r="O107" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P107" s="44" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="Q107" s="21">
         <f t="shared" ref="Q107" si="94">P107*N107</f>
@@ -8580,13 +8582,13 @@
         <v>401</v>
       </c>
       <c r="I108" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J108" s="14" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="K108" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L108" s="14">
         <v>1</v>
@@ -8599,10 +8601,10 @@
         <v>10</v>
       </c>
       <c r="O108" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P108" s="44" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="Q108" s="15">
         <f>P108*N108</f>
@@ -8635,13 +8637,13 @@
         <v>399</v>
       </c>
       <c r="I109" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J109" s="20" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="K109" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L109" s="20">
         <v>1</v>
@@ -8654,10 +8656,10 @@
         <v>10</v>
       </c>
       <c r="O109" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P109" s="44" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="Q109" s="21">
         <f t="shared" ref="Q109" si="96">P109*N109</f>
@@ -8690,13 +8692,13 @@
         <v>380</v>
       </c>
       <c r="I110" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J110" s="14" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="K110" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L110" s="14">
         <v>1</v>
@@ -8709,10 +8711,10 @@
         <v>6</v>
       </c>
       <c r="O110" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P110" s="44" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="Q110" s="15">
         <f>P110*N110</f>
@@ -8745,13 +8747,13 @@
         <v>402</v>
       </c>
       <c r="I111" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J111" s="20" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="K111" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L111" s="20">
         <v>1</v>
@@ -8764,10 +8766,10 @@
         <v>6</v>
       </c>
       <c r="O111" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P111" s="44" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="Q111" s="21">
         <f t="shared" ref="Q111" si="98">P111*N111</f>
@@ -8800,13 +8802,13 @@
         <v>398</v>
       </c>
       <c r="I112" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J112" s="14" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="K112" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L112" s="14">
         <v>1</v>
@@ -8819,10 +8821,10 @@
         <v>10</v>
       </c>
       <c r="O112" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P112" s="44" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="Q112" s="15">
         <f>P112*N112</f>
@@ -8846,7 +8848,7 @@
         <v>235</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>369</v>
@@ -8855,13 +8857,13 @@
         <v>403</v>
       </c>
       <c r="I113" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J113" s="20" t="s">
+        <v>500</v>
+      </c>
+      <c r="K113" s="20" t="s">
         <v>501</v>
-      </c>
-      <c r="K113" s="20" t="s">
-        <v>502</v>
       </c>
       <c r="L113" s="20">
         <v>1</v>
@@ -8871,13 +8873,13 @@
         <v>5</v>
       </c>
       <c r="N113" s="14" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="O113" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P113" s="44" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="Q113" s="21">
         <f t="shared" ref="Q113" si="100">P113*N113</f>
@@ -8910,13 +8912,13 @@
         <v>404</v>
       </c>
       <c r="I114" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J114" s="14" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="K114" s="20" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L114" s="14">
         <v>1</v>
@@ -8929,7 +8931,7 @@
         <v>6</v>
       </c>
       <c r="O114" s="45" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="P114" s="44">
         <v>9.16</v>
@@ -8965,13 +8967,13 @@
         <v>405</v>
       </c>
       <c r="I115" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J115" s="20" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="K115" s="20" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="L115" s="20">
         <v>1</v>
@@ -8984,10 +8986,10 @@
         <v>10</v>
       </c>
       <c r="O115" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P115" s="44" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="Q115" s="21">
         <f t="shared" ref="Q115" si="102">P115*N115</f>
@@ -9011,7 +9013,7 @@
         <v>238</v>
       </c>
       <c r="F116" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G116" s="14" t="s">
         <v>372</v>
@@ -9020,13 +9022,13 @@
         <v>406</v>
       </c>
       <c r="I116" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J116" s="14" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="K116" s="14" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="L116" s="14">
         <v>1</v>
@@ -9036,13 +9038,13 @@
         <v>5</v>
       </c>
       <c r="N116" s="14" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="O116" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P116" s="44" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="Q116" s="15">
         <f>P116*N116</f>
@@ -9066,7 +9068,7 @@
         <v>239</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G117" s="20" t="s">
         <v>373</v>
@@ -9075,13 +9077,13 @@
         <v>407</v>
       </c>
       <c r="I117" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J117" s="20" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="K117" s="20" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="L117" s="20">
         <v>1</v>
@@ -9094,10 +9096,10 @@
         <v>6</v>
       </c>
       <c r="O117" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P117" s="44" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="Q117" s="21">
         <f t="shared" ref="Q117" si="104">P117*N117</f>
@@ -9130,13 +9132,13 @@
         <v>408</v>
       </c>
       <c r="I118" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J118" s="14" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="K118" s="14" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="L118" s="14">
         <v>1</v>
@@ -9149,10 +9151,10 @@
         <v>6</v>
       </c>
       <c r="O118" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P118" s="44" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="Q118" s="15">
         <f>P118*N118</f>
@@ -9185,13 +9187,13 @@
         <v>409</v>
       </c>
       <c r="I119" s="53" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="J119" s="20" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="K119" s="20" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="L119" s="20">
         <v>1</v>
@@ -9204,10 +9206,10 @@
         <v>6</v>
       </c>
       <c r="O119" s="45" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="P119" s="44" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="Q119" s="21">
         <f t="shared" ref="Q119" si="106">P119*N119</f>
@@ -9236,7 +9238,7 @@
       <c r="P120" s="57"/>
       <c r="Q120" s="18">
         <f>SUM(Q8:Q119)</f>
-        <v>480.49539999999996</v>
+        <v>477.55539999999991</v>
       </c>
       <c r="R120" s="1"/>
     </row>
@@ -9261,7 +9263,7 @@
       <c r="P121" s="57"/>
       <c r="Q121" s="19">
         <f>Q120/5</f>
-        <v>96.099079999999987</v>
+        <v>95.511079999999978</v>
       </c>
       <c r="R121" s="1"/>
     </row>
@@ -9386,8 +9388,9 @@
     <hyperlink ref="O111" r:id="rId109"/>
     <hyperlink ref="O112" r:id="rId110"/>
     <hyperlink ref="O114" r:id="rId111"/>
+    <hyperlink ref="O87" r:id="rId112"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId112"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId113"/>
 </worksheet>
 </file>
</xml_diff>